<commit_message>
Update: Threat Alert Report - 2026-03-23 09:33
</commit_message>
<xml_diff>
--- a/excel_routes/route_AHB_CAI_threats.xlsx
+++ b/excel_routes/route_AHB_CAI_threats.xlsx
@@ -33,7 +33,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -48,8 +48,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+        <bgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00D4EDDA"/>
         <bgColor rgb="00D4EDDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+        <bgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
   </fills>
@@ -71,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -80,6 +92,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -447,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -459,7 +477,7 @@
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -523,12 +541,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>01-MAR-26</t>
+          <t>26-MAR-26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SM-444</t>
+          <t>SM-448</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -537,13 +555,13 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>763</v>
+        <v>2071</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>883</v>
+        <v>2593</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-120</v>
+        <v>-522</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>30</v>
@@ -556,7 +574,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>HIGH THREAT ALERT - NEED ACTION</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -568,7 +586,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>01-MAR-26</t>
+          <t>27-MAR-26</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -582,13 +600,13 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>800</v>
+        <v>2394</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>883</v>
+        <v>2593</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-83</v>
+        <v>-199</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>30</v>
@@ -599,7 +617,7 @@
       <c r="I3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>LOW THREAT</t>
         </is>
@@ -613,12 +631,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>19-MAR-26</t>
+          <t>29-MAR-26</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SM-448</t>
+          <t>SM-444</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -627,13 +645,13 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1271</v>
+        <v>2071</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>1306</v>
+        <v>2593</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>-35</v>
+        <v>-522</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>30</v>
@@ -646,7 +664,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>HIGH THREAT ALERT - NEED ACTION</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -658,7 +676,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>20-MAR-26</t>
+          <t>30-MAR-26</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -672,119 +690,29 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1136</v>
+        <v>2389</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>1013</v>
+        <v>2593</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>123</v>
+        <v>-204</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>-10</v>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>LOW THREAT</t>
+        <v>0</v>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>SAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>26-MAR-26</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>SM-448</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Nile Air NP-144</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>640</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>648</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>-8</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>LOW THREAT</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>SAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>29-MAR-26</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>SM-444</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Nile Air NP-144</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>671</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>721</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>-50</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>LOW THREAT</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>SAR</t>
         </is>

</xml_diff>

<commit_message>
Update: Threat Alert Report - 2026-05-17 05:45
</commit_message>
<xml_diff>
--- a/excel_routes/route_AHB_CAI_threats.xlsx
+++ b/excel_routes/route_AHB_CAI_threats.xlsx
@@ -54,14 +54,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
-        <bgColor rgb="00FFF3CD"/>
+        <fgColor rgb="00F8D7DA"/>
+        <bgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
-        <bgColor rgb="00F8D7DA"/>
+        <fgColor rgb="00FFF3CD"/>
+        <bgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
   </fills>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>06-APR-26</t>
+          <t>20-MAY-26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -551,26 +551,26 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1140</v>
+        <v>1101</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1199</v>
+        <v>1368</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-59</v>
+        <v>-267</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>30</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
@@ -586,7 +586,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>06-APR-26</t>
+          <t>25-MAY-26</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -596,17 +596,17 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1140</v>
+        <v>1495</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1199</v>
+        <v>1947</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-59</v>
+        <v>-452</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>30</v>
@@ -617,9 +617,9 @@
       <c r="I3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>LOW THREAT</t>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>HIGH THREAT ALERT - NEED ACTION</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -631,7 +631,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>09-APR-26</t>
+          <t>25-MAY-26</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -641,17 +641,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-436</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>802</v>
+        <v>1895</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>826</v>
+        <v>1947</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>-24</v>
+        <v>-52</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>30</v>
@@ -676,7 +676,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>09-APR-26</t>
+          <t>25-MAY-26</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -686,17 +686,17 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>802</v>
+        <v>1935</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>826</v>
+        <v>1947</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-24</v>
+        <v>-12</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>30</v>
@@ -721,7 +721,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>11-APR-26</t>
+          <t>30-MAY-26</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -731,17 +731,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>677</v>
+        <v>763</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>826</v>
+        <v>783</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-149</v>
+        <v>-20</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>30</v>
@@ -766,7 +766,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>11-APR-26</t>
+          <t>01-JUN-26</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -776,26 +776,26 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>677</v>
+        <v>929</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>826</v>
+        <v>848</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-149</v>
+        <v>81</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>13-APR-26</t>
+          <t>10-JUN-26</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -821,17 +821,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>671</v>
+        <v>648</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>761</v>
+        <v>710</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-90</v>
+        <v>-62</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>30</v>
@@ -856,7 +856,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>13-APR-26</t>
+          <t>11-JUN-26</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -870,22 +870,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>671</v>
+        <v>912</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>761</v>
+        <v>783</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-90</v>
+        <v>129</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
@@ -901,7 +901,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>16-MAY-26</t>
+          <t>24-JUN-26</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -911,30 +911,30 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>1017</v>
+        <v>1271</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>1541</v>
+        <v>1368</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>-524</v>
+        <v>-97</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>30</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+        <v>0</v>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>16-MAY-26</t>
+          <t>25-JUN-26</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -956,30 +956,30 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1017</v>
+        <v>1545</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>1541</v>
+        <v>1563</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-524</v>
+        <v>-18</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>30</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+        <v>0</v>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -991,7 +991,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>18-MAY-26</t>
+          <t>01-JUL-26</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1001,30 +1001,30 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1012</v>
+        <v>1471</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1541</v>
+        <v>1563</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-529</v>
+        <v>-92</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>30</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+        <v>0</v>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>18-MAY-26</t>
+          <t>08-JUL-26</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1046,30 +1046,30 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1012</v>
+        <v>1271</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>1541</v>
+        <v>1368</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-529</v>
+        <v>-97</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>30</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+        <v>0</v>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1081,7 +1081,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>20-MAY-26</t>
+          <t>11-JUL-26</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1091,26 +1091,26 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1271</v>
+        <v>1068</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>1541</v>
+        <v>1368</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-270</v>
+        <v>-300</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>20-MAY-26</t>
+          <t>11-JUL-26</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1136,26 +1136,26 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>1271</v>
+        <v>1118</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>1541</v>
+        <v>1368</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-270</v>
+        <v>-250</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>21-MAY-26</t>
+          <t>11-JUL-26</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1181,26 +1181,26 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>1345</v>
+        <v>1118</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>1541</v>
+        <v>1368</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>-196</v>
+        <v>-250</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>21-MAY-26</t>
+          <t>11-JUL-26</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1226,26 +1226,26 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>1345</v>
+        <v>1118</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>1541</v>
+        <v>1368</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>-196</v>
+        <v>-250</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
@@ -1261,7 +1261,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>23-MAY-26</t>
+          <t>13-JUL-26</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1271,26 +1271,26 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>1350</v>
+        <v>1018</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>1541</v>
+        <v>1368</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>-191</v>
+        <v>-350</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
@@ -1306,7 +1306,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>23-MAY-26</t>
+          <t>13-JUL-26</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1316,26 +1316,26 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>1350</v>
+        <v>1063</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>1541</v>
+        <v>1368</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>-191</v>
+        <v>-305</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
@@ -1351,7 +1351,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>25-MAY-26</t>
+          <t>13-JUL-26</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1361,26 +1361,26 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>1345</v>
+        <v>1068</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>1541</v>
+        <v>1368</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>-196</v>
+        <v>-300</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H20" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
@@ -1396,7 +1396,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>25-MAY-26</t>
+          <t>13-JUL-26</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1406,17 +1406,17 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>1345</v>
+        <v>1185</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>1541</v>
+        <v>1368</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>-196</v>
+        <v>-183</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>30</v>
@@ -1441,7 +1441,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>01-JUN-26</t>
+          <t>13-JUL-26</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1451,17 +1451,17 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>727</v>
+        <v>1185</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>826</v>
+        <v>1368</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>-99</v>
+        <v>-183</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>30</v>
@@ -1486,7 +1486,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>01-JUN-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1496,26 +1496,26 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>727</v>
+        <v>1008</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>826</v>
+        <v>1368</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>-99</v>
+        <v>-360</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H23" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
@@ -1531,7 +1531,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>03-JUN-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1541,26 +1541,26 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>640</v>
+        <v>1018</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>826</v>
+        <v>1368</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>-186</v>
+        <v>-350</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H24" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
@@ -1576,7 +1576,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>03-JUN-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1586,26 +1586,26 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>640</v>
+        <v>1088</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>826</v>
+        <v>1368</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>-186</v>
+        <v>-280</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H25" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>04-JUN-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1631,17 +1631,17 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>727</v>
+        <v>1195</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>826</v>
+        <v>1368</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>-99</v>
+        <v>-173</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>30</v>
@@ -1666,7 +1666,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>04-JUN-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1676,17 +1676,17 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>727</v>
+        <v>1271</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>826</v>
+        <v>1368</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>-99</v>
+        <v>-97</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>30</v>
@@ -1711,7 +1711,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>06-JUN-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1721,14 +1721,14 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>733</v>
+        <v>1275</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>826</v>
+        <v>1368</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>-93</v>
@@ -1756,7 +1756,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>06-JUN-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1766,26 +1766,26 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>733</v>
+        <v>958</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>826</v>
+        <v>1368</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>-93</v>
+        <v>-410</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H29" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
@@ -1801,7 +1801,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>08-JUN-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1811,26 +1811,26 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>727</v>
+        <v>1058</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>826</v>
+        <v>1368</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>-99</v>
+        <v>-310</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H30" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
@@ -1846,7 +1846,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>08-JUN-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1860,22 +1860,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>727</v>
+        <v>1063</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>826</v>
+        <v>1368</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>-99</v>
+        <v>-305</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H31" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
@@ -1891,7 +1891,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>10-JUN-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1901,26 +1901,26 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>640</v>
+        <v>1118</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>826</v>
+        <v>1368</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>-186</v>
+        <v>-250</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H32" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
@@ -1936,7 +1936,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>10-JUN-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1946,26 +1946,26 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>640</v>
+        <v>1138</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>826</v>
+        <v>1368</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>-186</v>
+        <v>-230</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H33" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
@@ -1981,7 +1981,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>25-JUN-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1991,17 +1991,17 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>1345</v>
+        <v>1195</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1768</v>
+        <v>1368</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>-423</v>
+        <v>-173</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>30</v>
@@ -2012,9 +2012,9 @@
       <c r="I34" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J34" s="5" t="inlineStr">
-        <is>
-          <t>HIGH THREAT ALERT - NEED ACTION</t>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -2026,7 +2026,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>25-JUN-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2036,17 +2036,17 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>1345</v>
+        <v>905</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>1768</v>
+        <v>1368</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>-423</v>
+        <v>-463</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>30</v>
@@ -2057,7 +2057,7 @@
       <c r="I35" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J35" s="5" t="inlineStr">
+      <c r="J35" s="4" t="inlineStr">
         <is>
           <t>HIGH THREAT ALERT - NEED ACTION</t>
         </is>
@@ -2071,7 +2071,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>27-JUN-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2085,26 +2085,26 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>1350</v>
+        <v>1069</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>1768</v>
+        <v>1368</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>-418</v>
+        <v>-299</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H36" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" s="5" t="inlineStr">
-        <is>
-          <t>HIGH THREAT ALERT - NEED ACTION</t>
+        <v>10</v>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -2116,7 +2116,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>27-JUN-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2126,17 +2126,17 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>1350</v>
+        <v>1115</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>1768</v>
+        <v>1368</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>-418</v>
+        <v>-253</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>30</v>
@@ -2149,7 +2149,7 @@
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>HIGH THREAT ALERT - NEED ACTION</t>
+          <t>MEDIUM THREAT - MONITOR</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -2161,7 +2161,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>29-JUN-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2171,17 +2171,17 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>1345</v>
+        <v>1155</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>1768</v>
+        <v>1368</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>-423</v>
+        <v>-213</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>30</v>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>HIGH THREAT ALERT - NEED ACTION</t>
+          <t>MEDIUM THREAT - MONITOR</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -2206,7 +2206,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>29-JUN-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2216,17 +2216,17 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>1345</v>
+        <v>1155</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>1768</v>
+        <v>1368</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>-423</v>
+        <v>-213</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>30</v>
@@ -2239,10 +2239,910 @@
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>18-JUL-26</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>1155</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>-213</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>18-JUL-26</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-438</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>1315</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>-53</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-342</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>758</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>-610</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I42" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-338</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>758</v>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>-610</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H43" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I43" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J43" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>768</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>-600</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>878</v>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>-490</v>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H45" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I45" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>878</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>-490</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I46" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>938</v>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>-430</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I47" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>938</v>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>-430</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I48" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-438</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>988</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>-380</v>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I49" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Nile Air NP-144</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>1101</v>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>-267</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>758</v>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>-610</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H51" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I51" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Air Arabia Egypt E5-512</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>776</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>-592</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I52" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
           <t>HIGH THREAT ALERT - NEED ACTION</t>
         </is>
       </c>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-338</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>788</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>-580</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H53" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I53" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>918</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>-450</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I54" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>958</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>-410</v>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I55" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-342</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>965</v>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>-403</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>HIGH THREAT ALERT - NEED ACTION</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="n">
+        <v>978</v>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>-390</v>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H57" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I57" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>1195</v>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>-173</v>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H58" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-438</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>1215</v>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>-153</v>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H59" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
         <is>
           <t>SAR</t>
         </is>

</xml_diff>

<commit_message>
Update: Threat Alert Report - 2026-05-17 13:14
</commit_message>
<xml_diff>
--- a/excel_routes/route_AHB_CAI_threats.xlsx
+++ b/excel_routes/route_AHB_CAI_threats.xlsx
@@ -477,7 +477,7 @@
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -574,7 +574,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -619,7 +619,7 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>HIGH THREAT ALERT - NEED ACTION</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -1879,7 +1879,7 @@
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>HIGH THREAT ALERT - NEED ACTION</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -2509,7 +2509,7 @@
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
@@ -2734,7 +2734,7 @@
       </c>
       <c r="J50" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="J51" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
@@ -2824,7 +2824,7 @@
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>HIGH THREAT ALERT - NEED ACTION</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
@@ -2869,7 +2869,7 @@
       </c>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="J54" s="5" t="inlineStr">
         <is>
-          <t>MEDIUM THREAT - MONITOR</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="J56" s="4" t="inlineStr">
         <is>
-          <t>HIGH THREAT ALERT - NEED ACTION</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
@@ -3094,7 +3094,7 @@
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
@@ -3139,7 +3139,7 @@
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>LOW THREAT</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update: Threat Alert Report - 2026-05-18 00:09
</commit_message>
<xml_diff>
--- a/excel_routes/route_AHB_CAI_threats.xlsx
+++ b/excel_routes/route_AHB_CAI_threats.xlsx
@@ -54,14 +54,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
-        <bgColor rgb="00F8D7DA"/>
+        <fgColor rgb="00FFF3CD"/>
+        <bgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
-        <bgColor rgb="00FFF3CD"/>
+        <fgColor rgb="00F8D7DA"/>
+        <bgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
   </fills>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -555,13 +555,13 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1101</v>
+        <v>1271</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1368</v>
+        <v>1563</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-267</v>
+        <v>-292</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>30</v>
@@ -586,27 +586,27 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>25-MAY-26</t>
+          <t>24-MAY-26</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SM-444</t>
+          <t>SM-968</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1495</v>
+        <v>1271</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1947</v>
+        <v>1312</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-452</v>
+        <v>-41</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>30</v>
@@ -617,9 +617,9 @@
       <c r="I3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -641,17 +641,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-436</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1895</v>
+        <v>1495</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>1947</v>
+        <v>1502</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>-52</v>
+        <v>-7</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>30</v>
@@ -676,27 +676,27 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>25-MAY-26</t>
+          <t>27-MAY-26</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>SM-444</t>
+          <t>SM-968</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1935</v>
+        <v>863</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>1947</v>
+        <v>1221</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-12</v>
+        <v>-358</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>30</v>
@@ -707,9 +707,9 @@
       <c r="I5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -721,12 +721,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>30-MAY-26</t>
+          <t>27-MAY-26</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>SM-444</t>
+          <t>SM-968</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -735,13 +735,13 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>763</v>
+        <v>863</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>783</v>
+        <v>1075</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-20</v>
+        <v>-212</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>30</v>
@@ -752,9 +752,9 @@
       <c r="I6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -766,36 +766,36 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>01-JUN-26</t>
+          <t>27-MAY-26</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>SM-444</t>
+          <t>SM-968</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>929</v>
+        <v>1045</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>848</v>
+        <v>1221</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>81</v>
+        <v>-176</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
@@ -811,27 +811,27 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>10-JUN-26</t>
+          <t>27-MAY-26</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>SM-444</t>
+          <t>SM-968</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>648</v>
+        <v>1145</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>710</v>
+        <v>1221</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-62</v>
+        <v>-76</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>30</v>
@@ -856,36 +856,36 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>11-JUN-26</t>
+          <t>27-MAY-26</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>SM-444</t>
+          <t>SM-968</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>912</v>
+        <v>1045</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>783</v>
+        <v>1075</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>129</v>
+        <v>-30</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
@@ -901,7 +901,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>24-JUN-26</t>
+          <t>28-MAY-26</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -911,26 +911,26 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>1271</v>
+        <v>1011</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>1368</v>
+        <v>945</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>-97</v>
+        <v>66</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
@@ -946,7 +946,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>25-JUN-26</t>
+          <t>30-MAY-26</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -956,17 +956,17 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1545</v>
+        <v>763</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>1563</v>
+        <v>783</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-18</v>
+        <v>-20</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>30</v>
@@ -991,7 +991,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>01-JUL-26</t>
+          <t>10-JUN-26</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1005,13 +1005,13 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1471</v>
+        <v>648</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1563</v>
+        <v>653</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-92</v>
+        <v>-5</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>30</v>
@@ -1036,7 +1036,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>08-JUL-26</t>
+          <t>24-JUN-26</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1081,7 +1081,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>11-JUL-26</t>
+          <t>29-JUN-26</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1091,26 +1091,26 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-342</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1068</v>
+        <v>1315</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-300</v>
+        <v>-53</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>11-JUL-26</t>
+          <t>01-JUL-26</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1136,26 +1136,26 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>1118</v>
+        <v>1471</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>1368</v>
+        <v>1563</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-250</v>
+        <v>-92</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>11-JUL-26</t>
+          <t>08-JUL-26</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1181,26 +1181,26 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>1118</v>
+        <v>1271</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>-250</v>
+        <v>-97</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>11-JUL-26</t>
+          <t>13-JUL-26</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1226,17 +1226,17 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>1118</v>
+        <v>1008</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>-250</v>
+        <v>-360</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>15</v>
@@ -1271,17 +1271,17 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>1018</v>
+        <v>1008</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>-350</v>
+        <v>-360</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>15</v>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
@@ -1396,7 +1396,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>13-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1406,26 +1406,26 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>1185</v>
+        <v>988</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>-183</v>
+        <v>-380</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H21" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
@@ -1441,7 +1441,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>13-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1455,22 +1455,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>1185</v>
+        <v>1008</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>-183</v>
+        <v>-360</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H22" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
@@ -1496,17 +1496,17 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>1008</v>
+        <v>1018</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>-360</v>
+        <v>-350</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>15</v>
@@ -1545,13 +1545,13 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>1018</v>
+        <v>1068</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>-350</v>
+        <v>-300</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15</v>
@@ -1586,26 +1586,26 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>1088</v>
+        <v>1271</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>-280</v>
+        <v>-97</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H25" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
@@ -1631,17 +1631,17 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>1195</v>
+        <v>1275</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>-173</v>
+        <v>-93</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>30</v>
@@ -1666,7 +1666,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1676,26 +1676,26 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>1271</v>
+        <v>958</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>-97</v>
+        <v>-410</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H27" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
@@ -1711,7 +1711,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1721,26 +1721,26 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>1275</v>
+        <v>1063</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>-93</v>
+        <v>-305</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H28" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
@@ -1766,17 +1766,17 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>958</v>
+        <v>1068</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>-410</v>
+        <v>-300</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>15</v>
@@ -1815,22 +1815,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>1058</v>
+        <v>1285</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>-310</v>
+        <v>-83</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H30" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
@@ -1856,26 +1856,26 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>1063</v>
+        <v>1315</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>-305</v>
+        <v>-53</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H31" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
@@ -1905,22 +1905,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>1118</v>
+        <v>1345</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>-250</v>
+        <v>-23</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H32" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
@@ -1936,7 +1936,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1946,17 +1946,17 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>1138</v>
+        <v>728</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>-230</v>
+        <v>-640</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>15</v>
@@ -1967,9 +1967,9 @@
       <c r="I33" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J33" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -1981,7 +1981,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1991,30 +1991,30 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>1195</v>
+        <v>938</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>-173</v>
+        <v>-430</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H34" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>15</v>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -2036,30 +2036,30 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>905</v>
+        <v>938</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>-463</v>
+        <v>-430</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H35" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -2081,26 +2081,26 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>1069</v>
+        <v>978</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>-299</v>
+        <v>-390</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H36" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
@@ -2126,30 +2126,30 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>1115</v>
+        <v>978</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>-253</v>
+        <v>-390</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H37" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" s="5" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>15</v>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -2171,30 +2171,30 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>1155</v>
+        <v>978</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>-213</v>
+        <v>-390</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H38" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" s="5" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>15</v>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -2216,30 +2216,30 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>1155</v>
+        <v>1069</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>-213</v>
+        <v>-299</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H39" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" s="5" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>10</v>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
@@ -2251,7 +2251,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>18-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2261,30 +2261,30 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>1155</v>
+        <v>698</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>-213</v>
+        <v>-670</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H40" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -2296,7 +2296,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>18-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2306,30 +2306,30 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>flyadeal F3-342</t>
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>1315</v>
+        <v>758</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>-53</v>
+        <v>-610</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H41" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J41" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>15</v>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
@@ -2341,7 +2341,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-342</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
@@ -2372,7 +2372,7 @@
       <c r="I42" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J42" s="5" t="inlineStr">
+      <c r="J42" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2386,7 +2386,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2396,30 +2396,30 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>758</v>
+        <v>776</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>-610</v>
+        <v>-592</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H43" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
@@ -2431,7 +2431,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2441,17 +2441,17 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>768</v>
+        <v>878</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>-600</v>
+        <v>-490</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>15</v>
@@ -2462,7 +2462,7 @@
       <c r="I44" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J44" s="5" t="inlineStr">
+      <c r="J44" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2476,7 +2476,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D45" s="2" t="n">
@@ -2507,7 +2507,7 @@
       <c r="I45" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J45" s="5" t="inlineStr">
+      <c r="J45" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2521,7 +2521,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2531,17 +2531,17 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>878</v>
+        <v>898</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>-490</v>
+        <v>-470</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>15</v>
@@ -2552,7 +2552,7 @@
       <c r="I46" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J46" s="5" t="inlineStr">
+      <c r="J46" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2566,7 +2566,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2597,7 +2597,7 @@
       <c r="I47" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J47" s="5" t="inlineStr">
+      <c r="J47" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2611,7 +2611,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2642,7 +2642,7 @@
       <c r="I48" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J48" s="5" t="inlineStr">
+      <c r="J48" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2666,17 +2666,17 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>flyadeal F3-342</t>
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>988</v>
+        <v>758</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>-380</v>
+        <v>-610</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>15</v>
@@ -2687,9 +2687,9 @@
       <c r="I49" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J49" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
@@ -2711,28 +2711,28 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>1101</v>
+        <v>758</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>-267</v>
+        <v>-610</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H50" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J50" s="5" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2746,7 +2746,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>22-JUL-26</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2760,13 +2760,13 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>758</v>
+        <v>768</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>-610</v>
+        <v>-600</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>15</v>
@@ -2777,7 +2777,7 @@
       <c r="I51" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J51" s="5" t="inlineStr">
+      <c r="J51" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2791,7 +2791,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>22-JUL-26</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2801,30 +2801,30 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>776</v>
+        <v>878</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>-592</v>
+        <v>-490</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H52" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
@@ -2836,7 +2836,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>22-JUL-26</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2846,17 +2846,17 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>788</v>
+        <v>878</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>-580</v>
+        <v>-490</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>15</v>
@@ -2867,7 +2867,7 @@
       <c r="I53" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J53" s="5" t="inlineStr">
+      <c r="J53" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2881,7 +2881,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>22-JUL-26</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2891,17 +2891,17 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>918</v>
+        <v>898</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>-450</v>
+        <v>-470</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>15</v>
@@ -2912,7 +2912,7 @@
       <c r="I54" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J54" s="5" t="inlineStr">
+      <c r="J54" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2926,7 +2926,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>22-JUL-26</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2936,17 +2936,17 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>958</v>
+        <v>938</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>-410</v>
+        <v>-430</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>15</v>
@@ -2957,9 +2957,9 @@
       <c r="I55" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J55" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
@@ -2971,7 +2971,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>22-JUL-26</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2981,30 +2981,30 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-342</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>965</v>
+        <v>938</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>-403</v>
+        <v>-430</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H56" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J56" s="4" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
@@ -3016,7 +3016,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>22-JUL-26</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -3026,30 +3026,30 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>978</v>
+        <v>1101</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>-390</v>
+        <v>-267</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H57" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J57" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>0</v>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
@@ -3061,7 +3061,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>25-JUL-26</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -3071,30 +3071,30 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>1195</v>
+        <v>698</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>-173</v>
+        <v>-670</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H58" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>15</v>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
@@ -3106,7 +3106,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>25-JUL-26</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -3116,33 +3116,348 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
+          <t>flyadeal F3-338</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>758</v>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>-610</v>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H59" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I59" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Air Arabia Egypt E5-514</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>781</v>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>-587</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I60" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
           <t>flyadeal F3-438</t>
         </is>
       </c>
-      <c r="D59" s="2" t="n">
-        <v>1215</v>
-      </c>
-      <c r="E59" s="2" t="n">
-        <v>1368</v>
-      </c>
-      <c r="F59" s="2" t="n">
-        <v>-153</v>
-      </c>
-      <c r="G59" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H59" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I59" s="2" t="n">
+      <c r="D61" s="2" t="n">
+        <v>858</v>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>-510</v>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H61" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I61" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>908</v>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>-460</v>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I62" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-342</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>935</v>
+      </c>
+      <c r="E63" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>-433</v>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H63" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I63" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J59" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="K59" s="2" t="inlineStr">
+      <c r="J63" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>938</v>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>-430</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I64" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>1085</v>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>-283</v>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H65" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>1145</v>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>-223</v>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
         <is>
           <t>SAR</t>
         </is>

</xml_diff>

<commit_message>
Update: Threat Alert Report - 2026-05-20 01:21
</commit_message>
<xml_diff>
--- a/excel_routes/route_AHB_CAI_threats.xlsx
+++ b/excel_routes/route_AHB_CAI_threats.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -477,7 +477,7 @@
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -555,13 +555,13 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1271</v>
+        <v>1101</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1312</v>
+        <v>1143</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-41</v>
+        <v>-42</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>30</v>
@@ -574,7 +574,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -586,7 +586,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>25-MAY-26</t>
+          <t>30-MAY-26</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -596,30 +596,30 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1148</v>
+        <v>648</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1502</v>
+        <v>710</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-354</v>
+        <v>-62</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -631,7 +631,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>27-MAY-26</t>
+          <t>03-JUN-26</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -645,13 +645,13 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>763</v>
+        <v>571</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>848</v>
+        <v>626</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>-85</v>
+        <v>-55</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>30</v>
@@ -664,7 +664,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -676,12 +676,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>27-MAY-26</t>
+          <t>10-JUN-26</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>SM-968</t>
+          <t>SM-444</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -690,13 +690,13 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>763</v>
+        <v>571</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>1075</v>
+        <v>626</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-312</v>
+        <v>-55</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>30</v>
@@ -707,9 +707,9 @@
       <c r="I5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -721,40 +721,40 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>27-MAY-26</t>
+          <t>17-JUN-26</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>SM-968</t>
+          <t>SM-444</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>788</v>
+        <v>671</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1075</v>
+        <v>783</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-287</v>
+        <v>-112</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -766,27 +766,27 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>27-MAY-26</t>
+          <t>22-JUN-26</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>SM-968</t>
+          <t>SM-444</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>828</v>
+        <v>948</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1075</v>
+        <v>1221</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-247</v>
+        <v>-273</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>15</v>
@@ -799,7 +799,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>28-MAY-26</t>
+          <t>24-JUN-26</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -821,30 +821,30 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>719</v>
+        <v>1271</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>945</v>
+        <v>1368</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-226</v>
+        <v>-97</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -856,7 +856,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>10-JUN-26</t>
+          <t>29-JUN-26</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -866,30 +866,30 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-342</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>648</v>
+        <v>1138</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>653</v>
+        <v>1368</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-5</v>
+        <v>-230</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>17-JUN-26</t>
+          <t>01-JUL-26</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -915,13 +915,13 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>671</v>
+        <v>1271</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>783</v>
+        <v>1563</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>-112</v>
+        <v>-292</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>30</v>
@@ -932,9 +932,9 @@
       <c r="I10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>22-JUN-26</t>
+          <t>08-JUL-26</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -956,30 +956,30 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>948</v>
+        <v>1271</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>1221</v>
+        <v>1368</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-273</v>
+        <v>-97</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -991,7 +991,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>24-JUN-26</t>
+          <t>11-JUL-26</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1001,30 +1001,30 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1271</v>
+        <v>1118</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-97</v>
+        <v>-250</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>29-JUN-26</t>
+          <t>11-JUL-26</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1046,30 +1046,30 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-342</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1315</v>
+        <v>1118</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-53</v>
+        <v>-250</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1081,7 +1081,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>01-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1091,30 +1091,30 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1271</v>
+        <v>988</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>1563</v>
+        <v>1368</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-292</v>
+        <v>-380</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>15</v>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1126,7 +1126,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>08-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1136,30 +1136,30 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>1271</v>
+        <v>1008</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-97</v>
+        <v>-360</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1171,7 +1171,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>11-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1181,17 +1181,17 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>1118</v>
+        <v>1018</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>-250</v>
+        <v>-350</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>15</v>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1216,7 +1216,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>11-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1226,17 +1226,17 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>1118</v>
+        <v>1068</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>-250</v>
+        <v>-300</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>15</v>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1271,30 +1271,30 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>1271</v>
+        <v>1068</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>-97</v>
+        <v>-300</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1306,7 +1306,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>20-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1316,30 +1316,30 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>698</v>
+        <v>1271</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>-670</v>
+        <v>-97</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>0</v>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1351,7 +1351,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>20-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1361,17 +1361,17 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-342</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>758</v>
+        <v>728</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>-610</v>
+        <v>-640</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>15</v>
@@ -1382,9 +1382,9 @@
       <c r="I20" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>HIGH THREAT ALERT - NEED ACTION</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1396,7 +1396,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>20-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1406,17 +1406,17 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>758</v>
+        <v>878</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>-610</v>
+        <v>-490</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>15</v>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>MEDIUM THREAT - MONITOR</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>20-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1451,30 +1451,30 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>776</v>
+        <v>978</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>-592</v>
+        <v>-390</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H22" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J22" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>15</v>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1486,7 +1486,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>20-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1500,13 +1500,13 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>878</v>
+        <v>1018</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>-490</v>
+        <v>-350</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>15</v>
@@ -1517,9 +1517,9 @@
       <c r="I23" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -1531,7 +1531,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>20-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1545,13 +1545,13 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>878</v>
+        <v>1018</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>-490</v>
+        <v>-350</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15</v>
@@ -1562,9 +1562,9 @@
       <c r="I24" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -1576,7 +1576,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>20-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1586,30 +1586,30 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>898</v>
+        <v>1058</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>-470</v>
+        <v>-310</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H25" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>10</v>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -1621,7 +1621,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>20-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1631,17 +1631,17 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>938</v>
+        <v>1088</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>-430</v>
+        <v>-280</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>15</v>
@@ -1652,9 +1652,9 @@
       <c r="I26" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -1676,17 +1676,17 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>938</v>
+        <v>698</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>-430</v>
+        <v>-670</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>15</v>
@@ -1697,9 +1697,9 @@
       <c r="I27" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>HIGH THREAT ALERT - NEED ACTION</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -1711,7 +1711,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1721,30 +1721,30 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-342</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>671</v>
+        <v>758</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>-697</v>
+        <v>-610</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H28" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>15</v>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -1756,7 +1756,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>MEDIUM THREAT - MONITOR</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -1801,7 +1801,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1811,30 +1811,30 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-342</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>788</v>
+        <v>768</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>-580</v>
+        <v>-600</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H30" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J30" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>10</v>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>HIGH THREAT ALERT - NEED ACTION</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -1846,7 +1846,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1856,17 +1856,17 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>788</v>
+        <v>878</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>-580</v>
+        <v>-490</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>15</v>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>MEDIUM THREAT - MONITOR</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -1891,7 +1891,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1901,17 +1901,17 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>898</v>
+        <v>878</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>-470</v>
+        <v>-490</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>15</v>
@@ -1924,7 +1924,7 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>MEDIUM THREAT - MONITOR</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -1936,7 +1936,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1946,17 +1946,17 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>918</v>
+        <v>938</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>-450</v>
+        <v>-430</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>15</v>
@@ -1969,7 +1969,7 @@
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>MEDIUM THREAT - MONITOR</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -1981,7 +1981,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1991,17 +1991,17 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>978</v>
+        <v>938</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>-390</v>
+        <v>-430</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>15</v>
@@ -2012,9 +2012,9 @@
       <c r="I34" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -2026,7 +2026,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2036,17 +2036,17 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>1008</v>
+        <v>938</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>-360</v>
+        <v>-430</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>15</v>
@@ -2057,9 +2057,9 @@
       <c r="I35" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J35" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -2071,7 +2071,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>22-JUL-26</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2081,33 +2081,798 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
+          <t>Nile Air NP-144</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>671</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>-697</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>HIGH THREAT ALERT - NEED ACTION</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-342</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>758</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>-610</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-338</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>758</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>-610</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>768</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>-600</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
           <t>flyadeal F3-20</t>
         </is>
       </c>
-      <c r="D36" s="2" t="n">
-        <v>1068</v>
-      </c>
-      <c r="E36" s="2" t="n">
-        <v>1368</v>
-      </c>
-      <c r="F36" s="2" t="n">
-        <v>-300</v>
-      </c>
-      <c r="G36" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="H36" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I36" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J36" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="D40" s="2" t="n">
+        <v>878</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>-490</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>878</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>-490</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-438</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>938</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>-430</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I42" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>938</v>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>-430</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H43" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I43" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>938</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>-430</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>698</v>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>-670</v>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H45" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I45" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>HIGH THREAT ALERT - NEED ACTION</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-342</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>758</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>-610</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I46" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Air Arabia Egypt E5-514</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>774</v>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>-594</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I47" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>HIGH THREAT ALERT - NEED ACTION</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>908</v>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>-460</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I48" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>908</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>-460</v>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I49" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-338</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>935</v>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>-433</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>HIGH THREAT ALERT - NEED ACTION</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-438</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>938</v>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>-430</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H51" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I51" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>938</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>-430</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I52" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM THREAT - MONITOR</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>968</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>-400</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H53" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I53" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
         <is>
           <t>SAR</t>
         </is>

</xml_diff>

<commit_message>
Update: Threat Alert Report - 2026-05-21 20:48
</commit_message>
<xml_diff>
--- a/excel_routes/route_AHB_CAI_threats.xlsx
+++ b/excel_routes/route_AHB_CAI_threats.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -523,7 +523,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>24-MAY-26</t>
+          <t>27-MAY-26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -537,13 +537,13 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1101</v>
+        <v>863</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1143</v>
+        <v>945</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-42</v>
+        <v>-82</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>30</v>
@@ -568,7 +568,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>27-MAY-26</t>
+          <t>28-MAY-26</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -578,26 +578,26 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>763</v>
+        <v>675</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>783</v>
+        <v>848</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-20</v>
+        <v>-173</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
@@ -613,12 +613,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>27-MAY-26</t>
+          <t>30-MAY-26</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SM-968</t>
+          <t>SM-444</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -627,13 +627,13 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>763</v>
+        <v>648</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>848</v>
+        <v>653</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>-85</v>
+        <v>-5</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>30</v>
@@ -650,186 +650,6 @@
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>SAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>28-MAY-26</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>SM-444</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Air Arabia Egypt E5-512</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>675</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>848</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>-173</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>SAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>30-MAY-26</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>SM-444</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Nile Air NP-144</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>648</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>710</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>-62</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>SAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>03-JUN-26</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>SM-444</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Nile Air NP-144</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>571</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>626</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>-55</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>SAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>10-JUN-26</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>SM-444</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Nile Air NP-144</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>571</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>626</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>-55</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>SAR</t>
         </is>

</xml_diff>

<commit_message>
Update: Threat Alert Report - 2026-05-22 15:50
</commit_message>
<xml_diff>
--- a/excel_routes/route_AHB_CAI_threats.xlsx
+++ b/excel_routes/route_AHB_CAI_threats.xlsx
@@ -33,7 +33,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +50,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D4EDDA"/>
         <bgColor rgb="00D4EDDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+        <bgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+        <bgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
   </fills>
@@ -71,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -80,6 +92,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -447,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -523,36 +541,36 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>27-MAY-26</t>
+          <t>23-MAY-26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SM-968</t>
+          <t>SM-444</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>863</v>
+        <v>834</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>945</v>
+        <v>1143</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-82</v>
+        <v>-309</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
@@ -568,40 +586,40 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>28-MAY-26</t>
+          <t>24-MAY-26</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SM-444</t>
+          <t>SM-968</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>675</v>
+        <v>1101</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>848</v>
+        <v>1312</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-173</v>
+        <v>-211</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>0</v>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -613,43 +631,1528 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>27-MAY-26</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>SM-968</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>748</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>1075</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>-327</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>27-MAY-26</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>SM-968</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-338</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>828</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>1075</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>-247</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>27-MAY-26</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>SM-968</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Nile Air NP-144</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>863</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>1075</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>-212</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>27-MAY-26</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>SM-968</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Nile Air NP-144</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>863</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>945</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>-82</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>28-MAY-26</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Air Arabia Egypt E5-512</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>631</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>848</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>-217</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>30-MAY-26</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>SM-444</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Nile Air NP-144</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D9" s="2" t="n">
         <v>648</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E9" s="2" t="n">
         <v>653</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F9" s="2" t="n">
         <v>-5</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I4" s="2" t="n">
+      <c r="G9" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>17-JUN-26</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Nile Air NP-144</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>763</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>783</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>-20</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>22-JUN-26</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Air Arabia Egypt E5-512</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>768</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>1075</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>-307</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>27-JUN-26</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Air Arabia Egypt E5-514</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>998</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>-370</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>27-JUN-26</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>1138</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>-230</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>01-JUL-26</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Nile Air NP-144</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>1471</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>1563</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>-92</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>08-JUL-26</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Nile Air NP-144</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>1271</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>-97</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>11-JUL-26</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Air Arabia Egypt E5-514</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>998</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>-370</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>15-JUL-26</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Nile Air NP-144</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>1271</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>-97</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>16-JUL-26</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>978</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>-390</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>16-JUL-26</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Air Arabia Egypt E5-512</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>1053</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>-315</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>16-JUL-26</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>-290</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>16-JUL-26</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>1088</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>-280</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>16-JUL-26</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>1138</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>-230</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>18-JUL-26</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>748</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>-620</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>18-JUL-26</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>898</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>-470</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>18-JUL-26</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>998</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>-370</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>18-JUL-26</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>998</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>-370</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>18-JUL-26</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>998</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>-370</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>18-JUL-26</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Air Arabia Egypt E5-514</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>998</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>-370</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Nile Air NP-144</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>671</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>-697</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-342</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>778</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>-590</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-338</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>778</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>-590</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>788</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>-580</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>898</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>-470</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>898</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>-470</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>898</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>-470</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-438</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>958</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>-410</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>958</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>-410</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>SAR</t>
         </is>

</xml_diff>

<commit_message>
Update: Threat Alert Report - 2026-05-23 04:14
</commit_message>
<xml_diff>
--- a/excel_routes/route_AHB_CAI_threats.xlsx
+++ b/excel_routes/route_AHB_CAI_threats.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -555,13 +555,13 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>834</v>
+        <v>856</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>1143</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-309</v>
+        <v>-287</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>20</v>
@@ -600,13 +600,13 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1101</v>
+        <v>971</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1312</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-211</v>
+        <v>-341</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>30</v>
@@ -636,31 +636,31 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SM-968</t>
+          <t>SM-444</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>748</v>
+        <v>763</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>1075</v>
+        <v>848</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>-327</v>
+        <v>-85</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
@@ -686,26 +686,26 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>828</v>
+        <v>763</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>1075</v>
+        <v>945</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-247</v>
+        <v>-182</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
@@ -721,40 +721,40 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>27-MAY-26</t>
+          <t>28-MAY-26</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>SM-968</t>
+          <t>SM-444</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>863</v>
+        <v>920</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1075</v>
+        <v>848</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-212</v>
+        <v>72</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>-10</v>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -766,12 +766,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>27-MAY-26</t>
+          <t>30-MAY-26</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>SM-968</t>
+          <t>SM-444</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -780,13 +780,13 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>863</v>
+        <v>648</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>945</v>
+        <v>653</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-82</v>
+        <v>-5</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>30</v>
@@ -811,7 +811,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>28-MAY-26</t>
+          <t>17-JUN-26</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -821,26 +821,26 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>631</v>
+        <v>763</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>848</v>
+        <v>783</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-217</v>
+        <v>-20</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>30-MAY-26</t>
+          <t>18-JUN-26</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -866,26 +866,26 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>648</v>
+        <v>768</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>653</v>
+        <v>1075</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-5</v>
+        <v>-307</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
@@ -901,7 +901,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>17-JUN-26</t>
+          <t>18-JUN-26</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -911,26 +911,26 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>763</v>
+        <v>788</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>783</v>
+        <v>1075</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>-20</v>
+        <v>-287</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
@@ -991,7 +991,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>27-JUN-26</t>
+          <t>22-JUN-26</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1001,30 +1001,30 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>998</v>
+        <v>1045</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1368</v>
+        <v>1075</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-370</v>
+        <v>-30</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>0</v>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1046,30 +1046,30 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1138</v>
+        <v>998</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-230</v>
+        <v>-370</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>10</v>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1081,7 +1081,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>01-JUL-26</t>
+          <t>27-JUN-26</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1091,26 +1091,26 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1471</v>
+        <v>1138</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>1563</v>
+        <v>1368</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-92</v>
+        <v>-230</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>08-JUL-26</t>
+          <t>29-JUN-26</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1136,30 +1136,30 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>1271</v>
+        <v>993</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-97</v>
+        <v>-375</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>10</v>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1171,7 +1171,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>11-JUL-26</t>
+          <t>01-JUL-26</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1181,30 +1181,30 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>998</v>
+        <v>1471</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>1368</v>
+        <v>1563</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>-370</v>
+        <v>-92</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>0</v>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1216,7 +1216,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>04-JUL-26</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1226,30 +1226,30 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>1271</v>
+        <v>998</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>-97</v>
+        <v>-370</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>10</v>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1261,7 +1261,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>08-JUL-26</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1271,26 +1271,26 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>978</v>
+        <v>1271</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>-390</v>
+        <v>-97</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
@@ -1306,7 +1306,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>11-JUL-26</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1316,17 +1316,17 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>1053</v>
+        <v>998</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>-315</v>
+        <v>-370</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>20</v>
@@ -1337,9 +1337,9 @@
       <c r="I19" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1351,7 +1351,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>11-JUL-26</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1361,26 +1361,26 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>1078</v>
+        <v>1365</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>-290</v>
+        <v>-3</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H20" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
@@ -1396,7 +1396,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>11-JUL-26</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1406,26 +1406,26 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>1088</v>
+        <v>1365</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>-280</v>
+        <v>-3</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H21" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
@@ -1441,7 +1441,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>11-JUL-26</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1451,26 +1451,26 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>1138</v>
+        <v>1365</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>-230</v>
+        <v>-3</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H22" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
@@ -1486,7 +1486,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>18-JUL-26</t>
+          <t>13-JUL-26</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1496,26 +1496,26 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>748</v>
+        <v>993</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>-620</v>
+        <v>-375</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H23" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
@@ -1531,7 +1531,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>18-JUL-26</t>
+          <t>13-JUL-26</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1545,13 +1545,13 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>898</v>
+        <v>1028</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>-470</v>
+        <v>-340</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>15</v>
@@ -1562,9 +1562,9 @@
       <c r="I24" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -1576,7 +1576,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>18-JUL-26</t>
+          <t>13-JUL-26</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1590,22 +1590,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>998</v>
+        <v>1205</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>-370</v>
+        <v>-163</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H25" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>18-JUL-26</t>
+          <t>13-JUL-26</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1635,22 +1635,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>998</v>
+        <v>1205</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>-370</v>
+        <v>-163</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H26" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
@@ -1666,7 +1666,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>18-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1676,17 +1676,17 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>998</v>
+        <v>1028</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>-370</v>
+        <v>-340</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>15</v>
@@ -1711,7 +1711,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>18-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1721,30 +1721,30 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>998</v>
+        <v>1028</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>-370</v>
+        <v>-340</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H28" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>15</v>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -1756,7 +1756,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1766,30 +1766,30 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>671</v>
+        <v>1058</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>-697</v>
+        <v>-310</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H29" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>15</v>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -1801,7 +1801,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1811,17 +1811,17 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-342</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>778</v>
+        <v>1088</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>-590</v>
+        <v>-280</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>15</v>
@@ -1832,9 +1832,9 @@
       <c r="I30" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J30" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -1846,7 +1846,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1856,17 +1856,17 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>778</v>
+        <v>1088</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>-590</v>
+        <v>-280</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>15</v>
@@ -1877,9 +1877,9 @@
       <c r="I31" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J31" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -1891,7 +1891,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1901,30 +1901,30 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>788</v>
+        <v>1271</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>-580</v>
+        <v>-97</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H32" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>0</v>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -1936,7 +1936,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1946,30 +1946,30 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>898</v>
+        <v>1053</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>-470</v>
+        <v>-315</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H33" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J33" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>10</v>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -1981,7 +1981,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1991,26 +1991,26 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>898</v>
+        <v>1155</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>-470</v>
+        <v>-213</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H34" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
@@ -2026,7 +2026,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2036,30 +2036,30 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>898</v>
+        <v>1255</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>-470</v>
+        <v>-113</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H35" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J35" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>0</v>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -2071,7 +2071,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2081,26 +2081,26 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>958</v>
+        <v>1265</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>-410</v>
+        <v>-103</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H36" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
@@ -2116,43 +2116,1573 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
+          <t>16-JUL-26</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>1315</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>-53</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>16-JUL-26</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-438</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>1335</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>-33</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>18-JUL-26</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>748</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>-620</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>18-JUL-26</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>898</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>-470</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>18-JUL-26</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>998</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>-370</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>18-JUL-26</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>998</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>-370</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I42" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>18-JUL-26</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>998</v>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>-370</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H43" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I43" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>18-JUL-26</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Air Arabia Egypt E5-514</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>998</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>-370</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>20-JUL-26</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Air Arabia Egypt E5-512</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>768</v>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>-600</v>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H45" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I45" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>20-JUL-26</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>895</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>-473</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>20-JUL-26</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>958</v>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>-410</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I47" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>20-JUL-26</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-342</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>985</v>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>-383</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>20-JUL-26</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-338</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>985</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>-383</v>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>20-JUL-26</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>1075</v>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>-293</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>20-JUL-26</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>1075</v>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>-293</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H51" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>20-JUL-26</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>1075</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>-293</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>20-JUL-26</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-438</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>1135</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>-233</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H53" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
           <t>22-JUL-26</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>SM-444</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Nile Air NP-144</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>671</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>-697</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-338</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>778</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>-590</v>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I55" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>788</v>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>-580</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="n">
+        <v>898</v>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>-470</v>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H57" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I57" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>898</v>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>-470</v>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H58" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I58" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-342</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>955</v>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>-413</v>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H59" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-438</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>958</v>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>-410</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I60" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>flyadeal F3-28</t>
         </is>
       </c>
-      <c r="D37" s="2" t="n">
+      <c r="D61" s="2" t="n">
         <v>958</v>
       </c>
-      <c r="E37" s="2" t="n">
-        <v>1368</v>
-      </c>
-      <c r="F37" s="2" t="n">
+      <c r="E61" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F61" s="2" t="n">
         <v>-410</v>
       </c>
-      <c r="G37" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="H37" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I37" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J37" s="3" t="inlineStr">
+      <c r="G61" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H61" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I61" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>1075</v>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>-293</v>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Air Arabia Egypt E5-514</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>774</v>
+      </c>
+      <c r="E63" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>-594</v>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H63" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I63" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J63" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>895</v>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>-473</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-342</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>955</v>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>-413</v>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H65" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-338</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>955</v>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>-413</v>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-438</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>1055</v>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>-313</v>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H67" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>1105</v>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>-263</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>1105</v>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>-263</v>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H69" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>1135</v>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>-233</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H70" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>1165</v>
+      </c>
+      <c r="E71" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F71" s="2" t="n">
+        <v>-203</v>
+      </c>
+      <c r="G71" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H71" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
         <is>
           <t>SAR</t>
         </is>

</xml_diff>

<commit_message>
Update: Threat Alert Report - 2026-05-23 06:23
</commit_message>
<xml_diff>
--- a/excel_routes/route_AHB_CAI_threats.xlsx
+++ b/excel_routes/route_AHB_CAI_threats.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K71"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -991,7 +991,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>22-JUN-26</t>
+          <t>27-JUN-26</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1001,30 +1001,30 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1045</v>
+        <v>998</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1075</v>
+        <v>1368</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-30</v>
+        <v>-370</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>10</v>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1046,30 +1046,30 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>998</v>
+        <v>1315</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-370</v>
+        <v>-53</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>0</v>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1081,7 +1081,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>27-JUN-26</t>
+          <t>29-JUN-26</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1091,30 +1091,30 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1138</v>
+        <v>993</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-230</v>
+        <v>-375</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>10</v>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1136,30 +1136,30 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-342</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>993</v>
+        <v>1335</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-375</v>
+        <v>-33</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>0</v>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1261,7 +1261,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>08-JUL-26</t>
+          <t>06-JUL-26</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1271,30 +1271,30 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>1271</v>
+        <v>993</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>-97</v>
+        <v>-375</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>10</v>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1306,7 +1306,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>11-JUL-26</t>
+          <t>08-JUL-26</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1316,30 +1316,30 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>998</v>
+        <v>1271</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>-370</v>
+        <v>-97</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>0</v>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1361,30 +1361,30 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>1365</v>
+        <v>998</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>-3</v>
+        <v>-370</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H20" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>10</v>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
@@ -1451,7 +1451,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
@@ -1486,7 +1486,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>13-JUL-26</t>
+          <t>11-JUL-26</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1496,30 +1496,30 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>993</v>
+        <v>1365</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>-375</v>
+        <v>-3</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H23" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>0</v>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -1541,30 +1541,30 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>1028</v>
+        <v>993</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>-340</v>
+        <v>-375</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H24" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>10</v>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -1666,7 +1666,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>13-JUL-26</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1676,26 +1676,26 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>1028</v>
+        <v>1205</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>-340</v>
+        <v>-163</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H27" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
@@ -1711,7 +1711,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>13-JUL-26</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1721,26 +1721,26 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>1028</v>
+        <v>1365</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>-340</v>
+        <v>-3</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H28" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
@@ -1766,26 +1766,26 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1058</v>
+        <v>1205</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>-310</v>
+        <v>-163</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H29" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
@@ -1811,26 +1811,26 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>1088</v>
+        <v>1205</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>-280</v>
+        <v>-163</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H30" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
@@ -1856,26 +1856,26 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>1088</v>
+        <v>1235</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>-280</v>
+        <v>-133</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H31" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
@@ -1901,17 +1901,17 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>1271</v>
+        <v>1265</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>-97</v>
+        <v>-103</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>30</v>
@@ -1936,7 +1936,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1946,26 +1946,26 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>1053</v>
+        <v>1265</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>-315</v>
+        <v>-103</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H33" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
@@ -1981,7 +1981,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1991,17 +1991,17 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>1155</v>
+        <v>1271</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>-213</v>
+        <v>-97</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>30</v>
@@ -2012,9 +2012,9 @@
       <c r="I34" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J34" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -2036,26 +2036,26 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>1255</v>
+        <v>978</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>-113</v>
+        <v>-390</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H35" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
@@ -2081,26 +2081,26 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>1265</v>
+        <v>1053</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>-103</v>
+        <v>-315</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H36" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
@@ -2126,26 +2126,26 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>1315</v>
+        <v>1078</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>-53</v>
+        <v>-290</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H37" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
@@ -2171,26 +2171,26 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>1335</v>
+        <v>1088</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>-33</v>
+        <v>-280</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H38" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
@@ -2206,7 +2206,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>18-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2216,17 +2216,17 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>748</v>
+        <v>1138</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>-620</v>
+        <v>-230</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>15</v>
@@ -2237,9 +2237,9 @@
       <c r="I39" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J39" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
@@ -2261,17 +2261,17 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>898</v>
+        <v>748</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>-470</v>
+        <v>-620</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>15</v>
@@ -2306,17 +2306,17 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>998</v>
+        <v>898</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>-370</v>
+        <v>-470</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>15</v>
@@ -2327,9 +2327,9 @@
       <c r="I41" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J41" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D43" s="2" t="n">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D44" s="2" t="n">
@@ -2454,17 +2454,17 @@
         <v>-370</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H44" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J44" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>15</v>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>20-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2486,17 +2486,17 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>768</v>
+        <v>998</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>-600</v>
+        <v>-370</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>20</v>
@@ -2507,9 +2507,9 @@
       <c r="I45" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J45" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -2531,26 +2531,26 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>895</v>
+        <v>768</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>-473</v>
+        <v>-600</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H46" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
@@ -2576,17 +2576,17 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>958</v>
+        <v>778</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>-410</v>
+        <v>-590</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>15</v>
@@ -2597,9 +2597,9 @@
       <c r="I47" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J47" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -2621,17 +2621,17 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-342</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>985</v>
+        <v>895</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>-383</v>
+        <v>-473</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>30</v>
@@ -2642,9 +2642,9 @@
       <c r="I48" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J48" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
@@ -2666,17 +2666,17 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>flyadeal F3-342</t>
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>985</v>
+        <v>955</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>-383</v>
+        <v>-413</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>30</v>
@@ -2687,9 +2687,9 @@
       <c r="I49" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J49" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
@@ -2881,7 +2881,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2891,17 +2891,17 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>671</v>
+        <v>1135</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>-697</v>
+        <v>-233</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>30</v>
@@ -2912,9 +2912,9 @@
       <c r="I54" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J54" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
@@ -2936,30 +2936,30 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>778</v>
+        <v>671</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>-590</v>
+        <v>-697</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H55" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J55" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>0</v>
+      </c>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
@@ -2981,30 +2981,30 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>flyadeal F3-342</t>
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>788</v>
+        <v>955</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>-580</v>
+        <v>-413</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H56" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>0</v>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
@@ -3026,30 +3026,30 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>898</v>
+        <v>955</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>-470</v>
+        <v>-413</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H57" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J57" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>0</v>
+      </c>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
@@ -3071,30 +3071,30 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>898</v>
+        <v>965</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>-470</v>
+        <v>-403</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H58" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J58" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>0</v>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
@@ -3116,17 +3116,17 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-342</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>955</v>
+        <v>1075</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>-413</v>
+        <v>-293</v>
       </c>
       <c r="G59" s="2" t="n">
         <v>30</v>
@@ -3137,9 +3137,9 @@
       <c r="I59" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J59" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr">
@@ -3161,30 +3161,30 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>958</v>
+        <v>1075</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>-410</v>
+        <v>-293</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H60" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J60" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>0</v>
+      </c>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
@@ -3206,30 +3206,30 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>958</v>
+        <v>1075</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>-410</v>
+        <v>-293</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H61" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J61" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>0</v>
+      </c>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
@@ -3251,17 +3251,17 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>1075</v>
+        <v>1135</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>-293</v>
+        <v>-233</v>
       </c>
       <c r="G62" s="2" t="n">
         <v>30</v>
@@ -3286,7 +3286,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>25-JUL-26</t>
+          <t>22-JUL-26</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -3296,30 +3296,30 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>774</v>
+        <v>1135</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>-594</v>
+        <v>-233</v>
       </c>
       <c r="G63" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H63" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J63" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>0</v>
+      </c>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -3331,7 +3331,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>25-JUL-26</t>
+          <t>23-JUL-26</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3341,26 +3341,26 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>895</v>
+        <v>768</v>
       </c>
       <c r="E64" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>-473</v>
+        <v>-600</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H64" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J64" s="5" t="inlineStr">
         <is>
@@ -3376,7 +3376,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>25-JUL-26</t>
+          <t>23-JUL-26</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-342</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D65" s="2" t="n">
@@ -3421,7 +3421,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>25-JUL-26</t>
+          <t>23-JUL-26</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3431,17 +3431,17 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>flyadeal F3-342</t>
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>955</v>
+        <v>985</v>
       </c>
       <c r="E66" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>-413</v>
+        <v>-383</v>
       </c>
       <c r="G66" s="2" t="n">
         <v>30</v>
@@ -3452,9 +3452,9 @@
       <c r="I66" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J66" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr">
@@ -3466,7 +3466,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>25-JUL-26</t>
+          <t>23-JUL-26</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3476,17 +3476,17 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>1055</v>
+        <v>985</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>-313</v>
+        <v>-383</v>
       </c>
       <c r="G67" s="2" t="n">
         <v>30</v>
@@ -3511,7 +3511,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>25-JUL-26</t>
+          <t>23-JUL-26</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3521,17 +3521,17 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>1105</v>
+        <v>1095</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>-263</v>
+        <v>-273</v>
       </c>
       <c r="G68" s="2" t="n">
         <v>30</v>
@@ -3556,7 +3556,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>25-JUL-26</t>
+          <t>23-JUL-26</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3570,13 +3570,13 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>1105</v>
+        <v>1115</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>-263</v>
+        <v>-253</v>
       </c>
       <c r="G69" s="2" t="n">
         <v>30</v>
@@ -3601,7 +3601,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>25-JUL-26</t>
+          <t>23-JUL-26</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3615,13 +3615,13 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>1135</v>
+        <v>1175</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F70" s="2" t="n">
-        <v>-233</v>
+        <v>-193</v>
       </c>
       <c r="G70" s="2" t="n">
         <v>30</v>
@@ -3632,9 +3632,9 @@
       <c r="I70" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J70" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
@@ -3646,43 +3646,493 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>1205</v>
+      </c>
+      <c r="E71" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F71" s="2" t="n">
+        <v>-163</v>
+      </c>
+      <c r="G71" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H71" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>1265</v>
+      </c>
+      <c r="E72" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F72" s="2" t="n">
+        <v>-103</v>
+      </c>
+      <c r="G72" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H72" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
           <t>25-JUL-26</t>
         </is>
       </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>SM-444</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Air Arabia Egypt E5-514</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>774</v>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F73" s="2" t="n">
+        <v>-594</v>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H73" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I73" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J73" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-338</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>778</v>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>-590</v>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J74" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-438</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>878</v>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>-490</v>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H75" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I75" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J75" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>895</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>-473</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-342</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>955</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>-413</v>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H77" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>1105</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>-263</v>
+      </c>
+      <c r="G78" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>1105</v>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F79" s="2" t="n">
+        <v>-263</v>
+      </c>
+      <c r="G79" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H79" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>1135</v>
+      </c>
+      <c r="E80" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F80" s="2" t="n">
+        <v>-233</v>
+      </c>
+      <c r="G80" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H80" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J80" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
         <is>
           <t>flyadeal F3-20</t>
         </is>
       </c>
-      <c r="D71" s="2" t="n">
+      <c r="D81" s="2" t="n">
         <v>1165</v>
       </c>
-      <c r="E71" s="2" t="n">
-        <v>1368</v>
-      </c>
-      <c r="F71" s="2" t="n">
+      <c r="E81" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F81" s="2" t="n">
         <v>-203</v>
       </c>
-      <c r="G71" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H71" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I71" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J71" s="4" t="inlineStr">
+      <c r="G81" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H81" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="K71" s="2" t="inlineStr">
+      <c r="K81" s="2" t="inlineStr">
         <is>
           <t>SAR</t>
         </is>

</xml_diff>

<commit_message>
Update: Threat Alert Report - 2026-05-23 11:01
</commit_message>
<xml_diff>
--- a/excel_routes/route_AHB_CAI_threats.xlsx
+++ b/excel_routes/route_AHB_CAI_threats.xlsx
@@ -48,12 +48,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D4EDDA"/>
-        <bgColor rgb="00D4EDDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF3CD"/>
         <bgColor rgb="00FFF3CD"/>
       </patternFill>
@@ -62,6 +56,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F8D7DA"/>
         <bgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4EDDA"/>
+        <bgColor rgb="00D4EDDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K81"/>
+  <dimension ref="A1:K76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -541,40 +541,40 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>23-MAY-26</t>
+          <t>24-MAY-26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SM-444</t>
+          <t>SM-968</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>856</v>
+        <v>971</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1143</v>
+        <v>1312</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-287</v>
+        <v>-341</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -586,40 +586,40 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>24-MAY-26</t>
+          <t>25-MAY-26</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SM-968</t>
+          <t>SM-444</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>971</v>
+        <v>1258</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1312</v>
+        <v>2242</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-341</v>
+        <v>-984</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -631,7 +631,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>27-MAY-26</t>
+          <t>25-MAY-26</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -641,30 +641,30 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-436</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>763</v>
+        <v>1708</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>848</v>
+        <v>2242</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>-85</v>
+        <v>-534</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -676,40 +676,40 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>27-MAY-26</t>
+          <t>25-MAY-26</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>SM-968</t>
+          <t>SM-444</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>763</v>
+        <v>1748</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>945</v>
+        <v>2242</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-182</v>
+        <v>-494</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -721,7 +721,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>28-MAY-26</t>
+          <t>25-MAY-26</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -731,28 +731,28 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>920</v>
+        <v>1878</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>848</v>
+        <v>2242</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>72</v>
+        <v>-364</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>-10</v>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -766,7 +766,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>30-MAY-26</t>
+          <t>25-MAY-26</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -776,28 +776,28 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>648</v>
+        <v>1878</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>653</v>
+        <v>2242</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-5</v>
+        <v>-364</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -811,7 +811,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>17-JUN-26</t>
+          <t>25-MAY-26</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -821,28 +821,28 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>763</v>
+        <v>1878</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>783</v>
+        <v>2242</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-20</v>
+        <v>-364</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -856,7 +856,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>18-JUN-26</t>
+          <t>25-MAY-26</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -866,28 +866,28 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-18</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>768</v>
+        <v>1878</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1075</v>
+        <v>2242</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-307</v>
+        <v>-364</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -901,7 +901,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>18-JUN-26</t>
+          <t>25-MAY-26</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -911,17 +911,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>788</v>
+        <v>1878</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>1075</v>
+        <v>2242</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>-287</v>
+        <v>-364</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>15</v>
@@ -932,7 +932,7 @@
       <c r="I10" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -946,7 +946,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>22-JUN-26</t>
+          <t>27-MAY-26</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -956,28 +956,28 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>768</v>
+        <v>763</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>1075</v>
+        <v>848</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-307</v>
+        <v>-85</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -991,40 +991,40 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>27-JUN-26</t>
+          <t>27-MAY-26</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>SM-444</t>
+          <t>SM-968</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>998</v>
+        <v>763</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1368</v>
+        <v>945</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-370</v>
+        <v>-182</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>0</v>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>27-JUN-26</t>
+          <t>30-MAY-26</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1046,17 +1046,17 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1315</v>
+        <v>648</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>1368</v>
+        <v>653</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-53</v>
+        <v>-5</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>30</v>
@@ -1067,7 +1067,7 @@
       <c r="I13" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1081,7 +1081,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>29-JUN-26</t>
+          <t>17-JUN-26</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1091,30 +1091,30 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>993</v>
+        <v>763</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>1368</v>
+        <v>783</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-375</v>
+        <v>-20</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>0</v>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1126,7 +1126,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>29-JUN-26</t>
+          <t>18-JUN-26</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1136,28 +1136,28 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-342</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>1335</v>
+        <v>768</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>1368</v>
+        <v>1075</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-33</v>
+        <v>-307</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
+        <v>10</v>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1171,7 +1171,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>01-JUL-26</t>
+          <t>18-JUN-26</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1181,28 +1181,28 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>1471</v>
+        <v>788</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>1563</v>
+        <v>1075</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>-92</v>
+        <v>-287</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1216,7 +1216,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>04-JUL-26</t>
+          <t>22-JUN-26</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1226,17 +1226,17 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>998</v>
+        <v>768</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>1368</v>
+        <v>1075</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>-370</v>
+        <v>-307</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>20</v>
@@ -1247,9 +1247,9 @@
       <c r="I17" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1261,7 +1261,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>06-JUL-26</t>
+          <t>29-JUN-26</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1275,13 +1275,13 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>-375</v>
+        <v>-376</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>20</v>
@@ -1292,7 +1292,7 @@
       <c r="I18" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -1306,7 +1306,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>08-JUL-26</t>
+          <t>01-JUL-26</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1320,13 +1320,13 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>1271</v>
+        <v>1471</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>1368</v>
+        <v>1563</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>-97</v>
+        <v>-92</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>30</v>
@@ -1337,7 +1337,7 @@
       <c r="I19" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J19" s="3" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1351,7 +1351,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>11-JUL-26</t>
+          <t>04-JUL-26</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1382,7 +1382,7 @@
       <c r="I20" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J20" s="4" t="inlineStr">
+      <c r="J20" s="3" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -1396,7 +1396,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>11-JUL-26</t>
+          <t>06-JUL-26</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1406,30 +1406,30 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>1365</v>
+        <v>992</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>-3</v>
+        <v>-376</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H21" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>11-JUL-26</t>
+          <t>08-JUL-26</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1451,17 +1451,17 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>1365</v>
+        <v>1271</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>-3</v>
+        <v>-97</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>30</v>
@@ -1472,7 +1472,7 @@
       <c r="I22" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J22" s="3" t="inlineStr">
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1496,30 +1496,30 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>1365</v>
+        <v>998</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>-3</v>
+        <v>-370</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H23" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -1531,7 +1531,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>13-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1541,30 +1541,30 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>993</v>
+        <v>1028</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>-375</v>
+        <v>-340</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H24" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>15</v>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -1576,7 +1576,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>13-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1586,28 +1586,28 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>1205</v>
+        <v>1028</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>-163</v>
+        <v>-340</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H25" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="3" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1621,7 +1621,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>13-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1631,28 +1631,28 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>1205</v>
+        <v>1058</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>-163</v>
+        <v>-310</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H26" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="3" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1666,7 +1666,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>13-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1676,28 +1676,28 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>1205</v>
+        <v>1088</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>-163</v>
+        <v>-280</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H27" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="3" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1711,7 +1711,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>13-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1725,24 +1725,24 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>1365</v>
+        <v>1088</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>-3</v>
+        <v>-280</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H28" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" s="3" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1766,17 +1766,17 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1205</v>
+        <v>1271</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>-163</v>
+        <v>-97</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>30</v>
@@ -1787,7 +1787,7 @@
       <c r="I29" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J29" s="3" t="inlineStr">
+      <c r="J29" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1801,7 +1801,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1815,24 +1815,24 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>1205</v>
+        <v>978</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>-163</v>
+        <v>-390</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H30" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="3" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1846,7 +1846,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1856,28 +1856,28 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>1235</v>
+        <v>1053</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>-133</v>
+        <v>-315</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H31" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" s="3" t="inlineStr">
+        <v>10</v>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1891,7 +1891,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1901,28 +1901,28 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>1265</v>
+        <v>1078</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>-103</v>
+        <v>-290</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H32" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" s="3" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J32" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1936,7 +1936,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1950,24 +1950,24 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>1265</v>
+        <v>1088</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>-103</v>
+        <v>-280</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H33" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" s="3" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -1981,7 +1981,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1991,28 +1991,28 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>1271</v>
+        <v>1138</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>-97</v>
+        <v>-230</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H34" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -2026,7 +2026,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2040,13 +2040,13 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>978</v>
+        <v>898</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>-390</v>
+        <v>-470</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>15</v>
@@ -2059,7 +2059,7 @@
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -2071,7 +2071,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2081,30 +2081,30 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>1053</v>
+        <v>925</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>-315</v>
+        <v>-443</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H36" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J36" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>0</v>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -2116,7 +2116,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2126,17 +2126,17 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>1078</v>
+        <v>998</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>-290</v>
+        <v>-370</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>15</v>
@@ -2147,7 +2147,7 @@
       <c r="I37" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J37" s="3" t="inlineStr">
+      <c r="J37" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -2161,7 +2161,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2171,17 +2171,17 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>1088</v>
+        <v>998</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>-280</v>
+        <v>-370</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>15</v>
@@ -2192,7 +2192,7 @@
       <c r="I38" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J38" s="3" t="inlineStr">
+      <c r="J38" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -2206,7 +2206,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2216,17 +2216,17 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>1138</v>
+        <v>998</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>-230</v>
+        <v>-370</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>15</v>
@@ -2237,7 +2237,7 @@
       <c r="I39" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J39" s="3" t="inlineStr">
+      <c r="J39" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -2261,28 +2261,28 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>748</v>
+        <v>998</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>-620</v>
+        <v>-370</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H40" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J40" s="4" t="inlineStr">
+        <v>10</v>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2296,7 +2296,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>18-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2306,30 +2306,30 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>898</v>
+        <v>768</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>-470</v>
+        <v>-600</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H41" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
@@ -2341,7 +2341,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>18-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2351,30 +2351,30 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>998</v>
+        <v>895</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>-370</v>
+        <v>-473</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H42" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J42" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>0</v>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -2386,7 +2386,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>18-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2396,30 +2396,30 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-342</t>
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>998</v>
+        <v>955</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>-370</v>
+        <v>-413</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H43" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J43" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>0</v>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
@@ -2431,7 +2431,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>18-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2441,30 +2441,30 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>998</v>
+        <v>955</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>-370</v>
+        <v>-413</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H44" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J44" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>0</v>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>18-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2486,30 +2486,30 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>998</v>
+        <v>958</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>-370</v>
+        <v>-410</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H45" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>15</v>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -2531,30 +2531,30 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>768</v>
+        <v>1075</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>-600</v>
+        <v>-293</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H46" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J46" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>0</v>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -2576,28 +2576,28 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>778</v>
+        <v>1075</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>-590</v>
+        <v>-293</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H47" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J47" s="4" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2621,17 +2621,17 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>895</v>
+        <v>1075</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>-473</v>
+        <v>-293</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>30</v>
@@ -2642,9 +2642,9 @@
       <c r="I48" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J48" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
@@ -2666,17 +2666,17 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-342</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>955</v>
+        <v>1135</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>-413</v>
+        <v>-233</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>30</v>
@@ -2687,9 +2687,9 @@
       <c r="I49" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J49" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
@@ -2701,7 +2701,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>20-JUL-26</t>
+          <t>22-JUL-26</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2711,17 +2711,17 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>1075</v>
+        <v>671</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>-293</v>
+        <v>-697</v>
       </c>
       <c r="G50" s="2" t="n">
         <v>30</v>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
@@ -2746,7 +2746,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>20-JUL-26</t>
+          <t>22-JUL-26</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2756,28 +2756,28 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-342</t>
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>1075</v>
+        <v>778</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>-293</v>
+        <v>-590</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H51" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J51" s="4" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2791,7 +2791,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>20-JUL-26</t>
+          <t>22-JUL-26</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2801,28 +2801,28 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>1075</v>
+        <v>778</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>-293</v>
+        <v>-590</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H52" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J52" s="4" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2836,7 +2836,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>20-JUL-26</t>
+          <t>22-JUL-26</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2846,28 +2846,28 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>1135</v>
+        <v>788</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>-233</v>
+        <v>-580</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H53" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J53" s="4" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2881,7 +2881,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>20-JUL-26</t>
+          <t>22-JUL-26</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2891,28 +2891,28 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>1135</v>
+        <v>898</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>-233</v>
+        <v>-470</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H54" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" s="4" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2936,30 +2936,30 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>671</v>
+        <v>898</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>-697</v>
+        <v>-470</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H55" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>15</v>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
@@ -2981,30 +2981,30 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-342</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>955</v>
+        <v>898</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>-413</v>
+        <v>-470</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H56" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J56" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>15</v>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
@@ -3026,30 +3026,30 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>955</v>
+        <v>958</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>-413</v>
+        <v>-410</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H57" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J57" s="5" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
@@ -3071,30 +3071,30 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>965</v>
+        <v>958</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>-403</v>
+        <v>-410</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H58" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J58" s="5" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
@@ -3106,7 +3106,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>23-JUL-26</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -3116,30 +3116,30 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>1075</v>
+        <v>768</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>-293</v>
+        <v>-600</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H59" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J59" s="4" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr">
@@ -3151,7 +3151,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>23-JUL-26</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -3161,17 +3161,17 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>1075</v>
+        <v>955</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>-293</v>
+        <v>-413</v>
       </c>
       <c r="G60" s="2" t="n">
         <v>30</v>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="J60" s="4" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
@@ -3196,7 +3196,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>23-JUL-26</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -3206,17 +3206,17 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-342</t>
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>1075</v>
+        <v>985</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>-293</v>
+        <v>-383</v>
       </c>
       <c r="G61" s="2" t="n">
         <v>30</v>
@@ -3227,7 +3227,7 @@
       <c r="I61" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J61" s="4" t="inlineStr">
+      <c r="J61" s="3" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3241,7 +3241,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>23-JUL-26</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3251,17 +3251,17 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>1135</v>
+        <v>985</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>-233</v>
+        <v>-383</v>
       </c>
       <c r="G62" s="2" t="n">
         <v>30</v>
@@ -3272,7 +3272,7 @@
       <c r="I62" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J62" s="4" t="inlineStr">
+      <c r="J62" s="3" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3286,7 +3286,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>23-JUL-26</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -3296,17 +3296,17 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>1135</v>
+        <v>1095</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>-233</v>
+        <v>-273</v>
       </c>
       <c r="G63" s="2" t="n">
         <v>30</v>
@@ -3317,7 +3317,7 @@
       <c r="I63" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J63" s="4" t="inlineStr">
+      <c r="J63" s="3" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3341,30 +3341,30 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>768</v>
+        <v>1115</v>
       </c>
       <c r="E64" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>-600</v>
+        <v>-253</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H64" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J64" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>0</v>
+      </c>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
@@ -3386,17 +3386,17 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>955</v>
+        <v>1175</v>
       </c>
       <c r="E65" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>-413</v>
+        <v>-193</v>
       </c>
       <c r="G65" s="2" t="n">
         <v>30</v>
@@ -3409,7 +3409,7 @@
       </c>
       <c r="J65" s="5" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
@@ -3431,17 +3431,17 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-342</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>985</v>
+        <v>1205</v>
       </c>
       <c r="E66" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>-383</v>
+        <v>-163</v>
       </c>
       <c r="G66" s="2" t="n">
         <v>30</v>
@@ -3452,9 +3452,9 @@
       <c r="I66" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J66" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr">
@@ -3476,17 +3476,17 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>985</v>
+        <v>1265</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>-383</v>
+        <v>-103</v>
       </c>
       <c r="G67" s="2" t="n">
         <v>30</v>
@@ -3497,9 +3497,9 @@
       <c r="I67" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J67" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J67" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr">
@@ -3511,7 +3511,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>25-JUL-26</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3521,30 +3521,30 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>1095</v>
+        <v>718</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>-273</v>
+        <v>-650</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H68" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J68" s="4" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
@@ -3556,7 +3556,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>25-JUL-26</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3566,30 +3566,30 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>1115</v>
+        <v>774</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>-253</v>
+        <v>-594</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H69" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J69" s="4" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr">
@@ -3601,7 +3601,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>25-JUL-26</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3611,30 +3611,30 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-342</t>
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>1175</v>
+        <v>778</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F70" s="2" t="n">
-        <v>-193</v>
+        <v>-590</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H70" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
@@ -3646,7 +3646,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>25-JUL-26</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -3656,30 +3656,30 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>1205</v>
+        <v>778</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>-163</v>
+        <v>-590</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H71" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
@@ -3691,7 +3691,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>25-JUL-26</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3701,30 +3701,30 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>1265</v>
+        <v>878</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F72" s="2" t="n">
-        <v>-103</v>
+        <v>-490</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H72" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -3746,30 +3746,30 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>774</v>
+        <v>928</v>
       </c>
       <c r="E73" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F73" s="2" t="n">
-        <v>-594</v>
+        <v>-440</v>
       </c>
       <c r="G73" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H73" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J73" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>15</v>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -3791,17 +3791,17 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>778</v>
+        <v>928</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F74" s="2" t="n">
-        <v>-590</v>
+        <v>-440</v>
       </c>
       <c r="G74" s="2" t="n">
         <v>15</v>
@@ -3812,7 +3812,7 @@
       <c r="I74" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J74" s="4" t="inlineStr">
+      <c r="J74" s="3" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3836,17 +3836,17 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>878</v>
+        <v>958</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F75" s="2" t="n">
-        <v>-490</v>
+        <v>-410</v>
       </c>
       <c r="G75" s="2" t="n">
         <v>15</v>
@@ -3857,9 +3857,9 @@
       <c r="I75" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J75" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J75" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K75" s="2" t="inlineStr">
@@ -3881,258 +3881,33 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>895</v>
+        <v>988</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F76" s="2" t="n">
-        <v>-473</v>
+        <v>-380</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H76" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J76" s="5" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr">
-        <is>
-          <t>SAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>25-JUL-26</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>SM-444</t>
-        </is>
-      </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>flyadeal F3-342</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="n">
-        <v>955</v>
-      </c>
-      <c r="E77" s="2" t="n">
-        <v>1368</v>
-      </c>
-      <c r="F77" s="2" t="n">
-        <v>-413</v>
-      </c>
-      <c r="G77" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H77" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J77" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="K77" s="2" t="inlineStr">
-        <is>
-          <t>SAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>25-JUL-26</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>SM-444</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>flyadeal F3-22</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="n">
-        <v>1105</v>
-      </c>
-      <c r="E78" s="2" t="n">
-        <v>1368</v>
-      </c>
-      <c r="F78" s="2" t="n">
-        <v>-263</v>
-      </c>
-      <c r="G78" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H78" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I78" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J78" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="K78" s="2" t="inlineStr">
-        <is>
-          <t>SAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>25-JUL-26</t>
-        </is>
-      </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t>SM-444</t>
-        </is>
-      </c>
-      <c r="C79" s="2" t="inlineStr">
-        <is>
-          <t>flyadeal F3-14</t>
-        </is>
-      </c>
-      <c r="D79" s="2" t="n">
-        <v>1105</v>
-      </c>
-      <c r="E79" s="2" t="n">
-        <v>1368</v>
-      </c>
-      <c r="F79" s="2" t="n">
-        <v>-263</v>
-      </c>
-      <c r="G79" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H79" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J79" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="K79" s="2" t="inlineStr">
-        <is>
-          <t>SAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>25-JUL-26</t>
-        </is>
-      </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>SM-444</t>
-        </is>
-      </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>flyadeal F3-28</t>
-        </is>
-      </c>
-      <c r="D80" s="2" t="n">
-        <v>1135</v>
-      </c>
-      <c r="E80" s="2" t="n">
-        <v>1368</v>
-      </c>
-      <c r="F80" s="2" t="n">
-        <v>-233</v>
-      </c>
-      <c r="G80" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H80" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I80" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J80" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="K80" s="2" t="inlineStr">
-        <is>
-          <t>SAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="2" t="inlineStr">
-        <is>
-          <t>25-JUL-26</t>
-        </is>
-      </c>
-      <c r="B81" s="2" t="inlineStr">
-        <is>
-          <t>SM-444</t>
-        </is>
-      </c>
-      <c r="C81" s="2" t="inlineStr">
-        <is>
-          <t>flyadeal F3-20</t>
-        </is>
-      </c>
-      <c r="D81" s="2" t="n">
-        <v>1165</v>
-      </c>
-      <c r="E81" s="2" t="n">
-        <v>1368</v>
-      </c>
-      <c r="F81" s="2" t="n">
-        <v>-203</v>
-      </c>
-      <c r="G81" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H81" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I81" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J81" s="4" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="K81" s="2" t="inlineStr">
         <is>
           <t>SAR</t>
         </is>

</xml_diff>

<commit_message>
Update: Threat Alert Report - 2026-06-03 11:22
</commit_message>
<xml_diff>
--- a/excel_routes/route_AHB_CAI_threats.xlsx
+++ b/excel_routes/route_AHB_CAI_threats.xlsx
@@ -54,14 +54,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
-        <bgColor rgb="00F8D7DA"/>
+        <fgColor rgb="00FFF3CD"/>
+        <bgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
-        <bgColor rgb="00FFF3CD"/>
+        <fgColor rgb="00F8D7DA"/>
+        <bgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
   </fills>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>03-JUN-26</t>
+          <t>10-JUN-26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -558,10 +558,10 @@
         <v>406</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>483</v>
+        <v>513</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-77</v>
+        <v>-107</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>30</v>
@@ -586,7 +586,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>10-JUN-26</t>
+          <t>17-JUN-26</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -600,13 +600,13 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>506</v>
+        <v>648</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>543</v>
+        <v>710</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-37</v>
+        <v>-62</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>30</v>
@@ -631,7 +631,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>17-JUN-26</t>
+          <t>20-JUN-26</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -641,26 +641,26 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>763</v>
+        <v>775</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>783</v>
+        <v>1075</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>-20</v>
+        <v>-300</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>18-JUN-26</t>
+          <t>20-JUN-26</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -686,26 +686,26 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>769</v>
+        <v>925</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>1075</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-306</v>
+        <v>-150</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>18-JUN-26</t>
+          <t>24-JUN-26</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -731,30 +731,30 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>828</v>
+        <v>863</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1075</v>
+        <v>1221</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-247</v>
+        <v>-358</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>0</v>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -766,7 +766,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>22-JUN-26</t>
+          <t>24-JUN-26</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -776,26 +776,26 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>769</v>
+        <v>918</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1075</v>
+        <v>1221</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-306</v>
+        <v>-303</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>24-JUN-26</t>
+          <t>27-JUN-26</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -821,26 +821,26 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1078</v>
+        <v>924</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>1368</v>
+        <v>1075</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-290</v>
+        <v>-151</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>24-JUN-26</t>
+          <t>29-JUN-26</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -866,26 +866,26 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>1271</v>
+        <v>919</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1368</v>
+        <v>1221</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-97</v>
+        <v>-302</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
@@ -901,7 +901,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>27-JUN-26</t>
+          <t>01-JUL-26</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -911,28 +911,28 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>999</v>
+        <v>1101</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>1563</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>-564</v>
+        <v>-462</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -946,7 +946,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>27-JUN-26</t>
+          <t>01-JUL-26</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -956,30 +956,30 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1098</v>
+        <v>1535</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>1563</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-465</v>
+        <v>-28</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>0</v>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -991,7 +991,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>29-JUN-26</t>
+          <t>02-JUL-26</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1005,13 +1005,13 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>994</v>
+        <v>1183</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1368</v>
+        <v>1563</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-374</v>
+        <v>-380</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>20</v>
@@ -1022,7 +1022,7 @@
       <c r="I12" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -1036,7 +1036,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>01-JUL-26</t>
+          <t>04-JUL-26</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1046,30 +1046,30 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1471</v>
+        <v>999</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>1563</v>
+        <v>1368</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-92</v>
+        <v>-369</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>10</v>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1081,7 +1081,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>08-JUL-26</t>
+          <t>06-JUL-26</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1091,28 +1091,28 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1101</v>
+        <v>994</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-267</v>
+        <v>-374</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="5" t="inlineStr">
+        <v>10</v>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -1126,7 +1126,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>11-JUL-26</t>
+          <t>08-JUL-26</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1136,28 +1136,28 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-514</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>999</v>
+        <v>971</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-369</v>
+        <v>-397</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -1181,30 +1181,30 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>1365</v>
+        <v>999</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>-3</v>
+        <v>-369</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>10</v>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1216,7 +1216,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>11-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1226,30 +1226,30 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>1365</v>
+        <v>938</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>-3</v>
+        <v>-430</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>15</v>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1261,7 +1261,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>13-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1271,17 +1271,17 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>978</v>
+        <v>938</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>-390</v>
+        <v>-430</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>15</v>
@@ -1292,9 +1292,9 @@
       <c r="I18" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1306,7 +1306,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>13-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1316,30 +1316,30 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>978</v>
+        <v>971</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>-390</v>
+        <v>-397</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>0</v>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1351,7 +1351,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>13-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1361,30 +1361,30 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>-374</v>
+        <v>-370</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H20" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>15</v>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1396,7 +1396,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>13-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1406,17 +1406,17 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>1028</v>
+        <v>1108</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>-340</v>
+        <v>-260</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>15</v>
@@ -1441,7 +1441,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>13-JUL-26</t>
+          <t>15-JUL-26</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1451,30 +1451,30 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>1088</v>
+        <v>1115</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>-280</v>
+        <v>-253</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H22" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>0</v>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1486,7 +1486,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1496,17 +1496,17 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>938</v>
+        <v>998</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>-430</v>
+        <v>-370</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>15</v>
@@ -1517,9 +1517,9 @@
       <c r="I23" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -1531,7 +1531,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1541,30 +1541,30 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>Air Arabia Egypt E5-512</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>971</v>
+        <v>1054</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>-397</v>
+        <v>-314</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H24" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>10</v>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -1576,7 +1576,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1586,30 +1586,30 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>1028</v>
+        <v>1115</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>-340</v>
+        <v>-253</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H25" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J25" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>0</v>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -1621,7 +1621,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>16-JUL-26</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1631,26 +1631,26 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>1028</v>
+        <v>1285</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>-340</v>
+        <v>-83</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H26" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
@@ -1666,7 +1666,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1676,17 +1676,17 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>1038</v>
+        <v>768</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>-330</v>
+        <v>-600</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>15</v>
@@ -1697,9 +1697,9 @@
       <c r="I27" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J27" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -1711,7 +1711,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>15-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1721,17 +1721,17 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>1108</v>
+        <v>978</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>-260</v>
+        <v>-390</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>15</v>
@@ -1756,7 +1756,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1766,17 +1766,17 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>938</v>
+        <v>998</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>-430</v>
+        <v>-370</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>15</v>
@@ -1787,9 +1787,9 @@
       <c r="I29" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J29" s="5" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -1801,7 +1801,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1811,17 +1811,17 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>1038</v>
+        <v>998</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>-330</v>
+        <v>-370</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>15</v>
@@ -1846,7 +1846,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1856,17 +1856,17 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Air Arabia Egypt E5-512</t>
+          <t>Air Arabia Egypt E5-514</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>1054</v>
+        <v>999</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>-314</v>
+        <v>-369</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>20</v>
@@ -1877,9 +1877,9 @@
       <c r="I31" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -1891,7 +1891,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1901,26 +1901,26 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>1255</v>
+        <v>1008</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>-113</v>
+        <v>-360</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H32" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
@@ -1936,7 +1936,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>16-JUL-26</t>
+          <t>18-JUL-26</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1946,26 +1946,26 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>1315</v>
+        <v>1038</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>-53</v>
+        <v>-330</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H33" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
@@ -1981,7 +1981,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>22-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1991,28 +1991,28 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-144</t>
+          <t>flyadeal F3-342</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>671</v>
+        <v>738</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>-697</v>
+        <v>-630</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H34" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2026,7 +2026,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2057,7 +2057,7 @@
       <c r="I35" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J35" s="4" t="inlineStr">
+      <c r="J35" s="5" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2071,7 +2071,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-346</t>
+          <t>flyadeal F3-338</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
@@ -2102,7 +2102,7 @@
       <c r="I36" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J36" s="5" t="inlineStr">
+      <c r="J36" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2116,7 +2116,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2126,30 +2126,30 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-338</t>
+          <t>flyadeal F3-346</t>
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>808</v>
+        <v>895</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>-560</v>
+        <v>-473</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H37" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -2161,7 +2161,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2171,28 +2171,28 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-342</t>
+          <t>flyadeal F3-438</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>985</v>
+        <v>918</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>-383</v>
+        <v>-450</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H38" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" s="5" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2206,7 +2206,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2216,30 +2216,30 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-438</t>
+          <t>flyadeal F3-28</t>
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>1095</v>
+        <v>998</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>-273</v>
+        <v>-370</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H39" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" s="5" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>15</v>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
@@ -2251,7 +2251,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2261,17 +2261,17 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-14</t>
+          <t>flyadeal F3-20</t>
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>1115</v>
+        <v>1075</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>-253</v>
+        <v>-293</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>30</v>
@@ -2282,7 +2282,7 @@
       <c r="I40" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J40" s="5" t="inlineStr">
+      <c r="J40" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2296,7 +2296,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2306,17 +2306,17 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-28</t>
+          <t>flyadeal F3-22</t>
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>1135</v>
+        <v>1075</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>-233</v>
+        <v>-293</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>30</v>
@@ -2327,7 +2327,7 @@
       <c r="I41" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="5" t="inlineStr">
+      <c r="J41" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2341,7 +2341,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>20-JUL-26</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2351,17 +2351,17 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-22</t>
+          <t>flyadeal F3-14</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>1155</v>
+        <v>1115</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>-213</v>
+        <v>-253</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>30</v>
@@ -2372,7 +2372,7 @@
       <c r="I42" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J42" s="5" t="inlineStr">
+      <c r="J42" s="4" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -2386,7 +2386,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>23-JUL-26</t>
+          <t>22-JUL-26</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2396,17 +2396,17 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>flyadeal F3-20</t>
+          <t>Nile Air NP-144</t>
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>1215</v>
+        <v>671</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>1368</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>-153</v>
+        <v>-697</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>30</v>
@@ -2417,12 +2417,1182 @@
       <c r="I43" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J43" s="3" t="inlineStr">
+      <c r="J43" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-342</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>748</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>-620</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-338</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>748</v>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>-620</v>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H45" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I45" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>758</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>-610</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I46" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>898</v>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>-470</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I47" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-438</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>918</v>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>-450</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I48" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>938</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>-430</v>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I49" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>938</v>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>-430</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I50" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>22-JUL-26</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>958</v>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>-410</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H51" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I51" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="K43" s="2" t="inlineStr">
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Air Arabia Egypt E5-512</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>769</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>-599</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I52" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>955</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>-413</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H53" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-342</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>985</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>-383</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-338</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>1025</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>-343</v>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-438</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>1095</v>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>-273</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="n">
+        <v>1115</v>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>-253</v>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H57" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>1175</v>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>-193</v>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H58" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>1205</v>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>-163</v>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H59" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>23-JUL-26</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>1265</v>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>-103</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="n">
+        <v>688</v>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>-680</v>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H61" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I61" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J61" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Air Arabia Egypt E5-514</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>775</v>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>-593</v>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I62" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J62" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-342</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>778</v>
+      </c>
+      <c r="E63" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>-590</v>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H63" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I63" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-338</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>778</v>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>-590</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I64" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-438</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>878</v>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>-490</v>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H65" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I65" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J65" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-22</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>888</v>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>-480</v>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I66" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-20</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>918</v>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>-450</v>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H67" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I67" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-14</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>928</v>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>-440</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I68" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J68" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>25-JUL-26</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>SM-444</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-28</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>958</v>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>1368</v>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>-410</v>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H69" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I69" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
         <is>
           <t>SAR</t>
         </is>

</xml_diff>